<commit_message>
Add By Subject sheet with color-coded Olympiad selections
- Preserved user's color coding for each student's selected subject
- Added "By Subject" sheet grouping all 42 students by their assigned subject
- Mathematics (15), Physics (6), English (8), Biology (4), Chemistry (2), IT (3), History (2), Not Assigned (2)
- Includes subject summary table with color legend
- Fixed Muhammad Yosin selection to Physics (yellow)

Co-Authored-By: Claude Opus 4.6 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01P4XDYqnEoWzCj2M7bmaBHG
</commit_message>
<xml_diff>
--- a/Ellipse_Olympiad_Students.xlsx
+++ b/Ellipse_Olympiad_Students.xlsx
@@ -13,6 +13,7 @@
     <sheet name="Grade 9" sheetId="4" state="visible" r:id="rId4"/>
     <sheet name="Grade 10" sheetId="5" state="visible" r:id="rId5"/>
     <sheet name="Grade 11" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet name="By Subject" sheetId="7" state="visible" r:id="rId7"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -22,7 +23,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="6">
+  <fonts count="10">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -56,8 +57,31 @@
       <color rgb="00333333"/>
       <sz val="11"/>
     </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <color rgb="00FFFFFF"/>
+      <sz val="12"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <color rgb="00666666"/>
+      <sz val="12"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <color rgb="00999999"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <color rgb="001F4E79"/>
+      <sz val="12"/>
+    </font>
   </fonts>
-  <fills count="5">
+  <fills count="13">
     <fill>
       <patternFill/>
     </fill>
@@ -80,6 +104,54 @@
       <patternFill patternType="solid">
         <fgColor rgb="00FFF2CC"/>
         <bgColor rgb="00FFF2CC"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FFC000"/>
+        <bgColor rgb="00FFC000"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FFFF00"/>
+        <bgColor rgb="00FFFF00"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="0092D050"/>
+        <bgColor rgb="0092D050"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="0000B0F0"/>
+        <bgColor rgb="0000B0F0"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00BF8F00"/>
+        <bgColor rgb="00BF8F00"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FF0000"/>
+        <bgColor rgb="00FF0000"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="007030A0"/>
+        <bgColor rgb="007030A0"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00F2F2F2"/>
+        <bgColor rgb="00F2F2F2"/>
       </patternFill>
     </fill>
   </fills>
@@ -109,7 +181,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="15">
+  <cellXfs count="43">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -134,6 +206,7 @@
     <xf numFmtId="49" fontId="3" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="3" fillId="5" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="5" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
@@ -142,7 +215,34 @@
     <xf numFmtId="49" fontId="3" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="3" fillId="6" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="7" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="8" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="9" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="10" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="11" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="6" fillId="5" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="6" fillId="6" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="6" fillId="7" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="6" fillId="8" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="6" fillId="10" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="6" fillId="11" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="6" fillId="9" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="7" fillId="12" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="8" fillId="12" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="8" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="10" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="11" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="9" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="12" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="4" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -708,7 +808,7 @@
           <t>7-P</t>
         </is>
       </c>
-      <c r="D4" s="8" t="inlineStr">
+      <c r="D4" s="10" t="inlineStr">
         <is>
           <t>Mathematics</t>
         </is>
@@ -723,44 +823,44 @@
           <t>Physics</t>
         </is>
       </c>
-      <c r="G4" s="10" t="n"/>
-      <c r="H4" s="10" t="n"/>
+      <c r="G4" s="11" t="n"/>
+      <c r="H4" s="11" t="n"/>
     </row>
     <row r="5">
-      <c r="A5" s="11" t="n">
+      <c r="A5" s="12" t="n">
         <v>2</v>
       </c>
-      <c r="B5" s="12" t="inlineStr">
+      <c r="B5" s="13" t="inlineStr">
         <is>
           <t>Avazbek Mirzaazizov</t>
         </is>
       </c>
-      <c r="C5" s="13" t="inlineStr">
+      <c r="C5" s="14" t="inlineStr">
         <is>
           <t>7-A</t>
         </is>
       </c>
-      <c r="D5" s="12" t="inlineStr">
+      <c r="D5" s="15" t="inlineStr">
         <is>
           <t>Physics</t>
         </is>
       </c>
-      <c r="E5" s="12" t="inlineStr">
-        <is>
-          <t>Mathematics</t>
-        </is>
-      </c>
-      <c r="F5" s="12" t="inlineStr">
+      <c r="E5" s="13" t="inlineStr">
+        <is>
+          <t>Mathematics</t>
+        </is>
+      </c>
+      <c r="F5" s="13" t="inlineStr">
         <is>
           <t>Biology</t>
         </is>
       </c>
-      <c r="G5" s="12" t="inlineStr">
-        <is>
-          <t>English</t>
-        </is>
-      </c>
-      <c r="H5" s="12" t="inlineStr">
+      <c r="G5" s="13" t="inlineStr">
+        <is>
+          <t>English</t>
+        </is>
+      </c>
+      <c r="H5" s="13" t="inlineStr">
         <is>
           <t>Chemistry</t>
         </is>
@@ -780,7 +880,7 @@
           <t>7-A</t>
         </is>
       </c>
-      <c r="D6" s="8" t="inlineStr">
+      <c r="D6" s="10" t="inlineStr">
         <is>
           <t>Mathematics</t>
         </is>
@@ -795,44 +895,44 @@
           <t>Biology</t>
         </is>
       </c>
-      <c r="G6" s="10" t="n"/>
-      <c r="H6" s="10" t="n"/>
+      <c r="G6" s="11" t="n"/>
+      <c r="H6" s="11" t="n"/>
     </row>
     <row r="7">
-      <c r="A7" s="11" t="n">
+      <c r="A7" s="12" t="n">
         <v>4</v>
       </c>
-      <c r="B7" s="12" t="inlineStr">
+      <c r="B7" s="13" t="inlineStr">
         <is>
           <t>Uzakbaev Imon</t>
         </is>
       </c>
-      <c r="C7" s="13" t="inlineStr">
+      <c r="C7" s="14" t="inlineStr">
         <is>
           <t>7-B</t>
         </is>
       </c>
-      <c r="D7" s="12" t="inlineStr">
-        <is>
-          <t>English</t>
-        </is>
-      </c>
-      <c r="E7" s="12" t="inlineStr">
-        <is>
-          <t>Mathematics</t>
-        </is>
-      </c>
-      <c r="F7" s="12" t="inlineStr">
+      <c r="D7" s="16" t="inlineStr">
+        <is>
+          <t>English</t>
+        </is>
+      </c>
+      <c r="E7" s="13" t="inlineStr">
+        <is>
+          <t>Mathematics</t>
+        </is>
+      </c>
+      <c r="F7" s="13" t="inlineStr">
         <is>
           <t>ICT</t>
         </is>
       </c>
-      <c r="G7" s="12" t="inlineStr">
+      <c r="G7" s="13" t="inlineStr">
         <is>
           <t>Biology</t>
         </is>
       </c>
-      <c r="H7" s="14" t="n"/>
+      <c r="H7" s="17" t="n"/>
     </row>
     <row r="8">
       <c r="A8" s="7" t="n">
@@ -853,7 +953,7 @@
           <t>Mathematics</t>
         </is>
       </c>
-      <c r="E8" s="8" t="inlineStr">
+      <c r="E8" s="15" t="inlineStr">
         <is>
           <t>Physics</t>
         </is>
@@ -863,36 +963,36 @@
           <t>English</t>
         </is>
       </c>
-      <c r="G8" s="10" t="n"/>
-      <c r="H8" s="10" t="n"/>
+      <c r="G8" s="11" t="n"/>
+      <c r="H8" s="11" t="n"/>
     </row>
     <row r="9">
-      <c r="A9" s="11" t="n">
+      <c r="A9" s="12" t="n">
         <v>6</v>
       </c>
-      <c r="B9" s="12" t="inlineStr">
+      <c r="B9" s="13" t="inlineStr">
         <is>
           <t>Kulboeva Medina-Aisha</t>
         </is>
       </c>
-      <c r="C9" s="13" t="inlineStr">
+      <c r="C9" s="14" t="inlineStr">
         <is>
           <t>7-P</t>
         </is>
       </c>
-      <c r="D9" s="12" t="inlineStr">
-        <is>
-          <t>Mathematics</t>
-        </is>
-      </c>
-      <c r="E9" s="12" t="inlineStr">
-        <is>
-          <t>English</t>
-        </is>
-      </c>
-      <c r="F9" s="14" t="n"/>
-      <c r="G9" s="14" t="n"/>
-      <c r="H9" s="14" t="n"/>
+      <c r="D9" s="10" t="inlineStr">
+        <is>
+          <t>Mathematics</t>
+        </is>
+      </c>
+      <c r="E9" s="13" t="inlineStr">
+        <is>
+          <t>English</t>
+        </is>
+      </c>
+      <c r="F9" s="17" t="n"/>
+      <c r="G9" s="17" t="n"/>
+      <c r="H9" s="17" t="n"/>
     </row>
     <row r="10">
       <c r="A10" s="7" t="n">
@@ -908,7 +1008,7 @@
           <t>7-P</t>
         </is>
       </c>
-      <c r="D10" s="8" t="inlineStr">
+      <c r="D10" s="10" t="inlineStr">
         <is>
           <t>Mathematics</t>
         </is>
@@ -918,9 +1018,9 @@
           <t>English</t>
         </is>
       </c>
-      <c r="F10" s="10" t="n"/>
-      <c r="G10" s="10" t="n"/>
-      <c r="H10" s="10" t="n"/>
+      <c r="F10" s="11" t="n"/>
+      <c r="G10" s="11" t="n"/>
+      <c r="H10" s="11" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="1">
@@ -1012,7 +1112,7 @@
           <t>8-B</t>
         </is>
       </c>
-      <c r="D4" s="8" t="inlineStr">
+      <c r="D4" s="18" t="inlineStr">
         <is>
           <t>Biology</t>
         </is>
@@ -1039,40 +1139,40 @@
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="11" t="n">
+      <c r="A5" s="12" t="n">
         <v>2</v>
       </c>
-      <c r="B5" s="12" t="inlineStr">
+      <c r="B5" s="13" t="inlineStr">
         <is>
           <t>Ziyodulla</t>
         </is>
       </c>
-      <c r="C5" s="13" t="inlineStr">
+      <c r="C5" s="14" t="inlineStr">
         <is>
           <t>8-G</t>
         </is>
       </c>
-      <c r="D5" s="12" t="inlineStr">
+      <c r="D5" s="19" t="inlineStr">
         <is>
           <t>History</t>
         </is>
       </c>
-      <c r="E5" s="12" t="inlineStr">
-        <is>
-          <t>Mathematics</t>
-        </is>
-      </c>
-      <c r="F5" s="12" t="inlineStr">
+      <c r="E5" s="13" t="inlineStr">
+        <is>
+          <t>Mathematics</t>
+        </is>
+      </c>
+      <c r="F5" s="13" t="inlineStr">
         <is>
           <t>Geography</t>
         </is>
       </c>
-      <c r="G5" s="12" t="inlineStr">
+      <c r="G5" s="13" t="inlineStr">
         <is>
           <t>Literature</t>
         </is>
       </c>
-      <c r="H5" s="12" t="inlineStr">
+      <c r="H5" s="13" t="inlineStr">
         <is>
           <t>English</t>
         </is>
@@ -1097,7 +1197,7 @@
           <t>English</t>
         </is>
       </c>
-      <c r="E6" s="8" t="inlineStr">
+      <c r="E6" s="18" t="inlineStr">
         <is>
           <t>Biology</t>
         </is>
@@ -1119,40 +1219,40 @@
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="11" t="n">
+      <c r="A7" s="12" t="n">
         <v>4</v>
       </c>
-      <c r="B7" s="12" t="inlineStr">
+      <c r="B7" s="13" t="inlineStr">
         <is>
           <t>Xasanova Latofat</t>
         </is>
       </c>
-      <c r="C7" s="13" t="inlineStr">
+      <c r="C7" s="14" t="inlineStr">
         <is>
           <t>8-P</t>
         </is>
       </c>
-      <c r="D7" s="12" t="inlineStr">
-        <is>
-          <t>Mathematics</t>
-        </is>
-      </c>
-      <c r="E7" s="12" t="inlineStr">
-        <is>
-          <t>English</t>
-        </is>
-      </c>
-      <c r="F7" s="12" t="inlineStr">
+      <c r="D7" s="10" t="inlineStr">
+        <is>
+          <t>Mathematics</t>
+        </is>
+      </c>
+      <c r="E7" s="13" t="inlineStr">
+        <is>
+          <t>English</t>
+        </is>
+      </c>
+      <c r="F7" s="13" t="inlineStr">
         <is>
           <t>Physics</t>
         </is>
       </c>
-      <c r="G7" s="12" t="inlineStr">
+      <c r="G7" s="13" t="inlineStr">
         <is>
           <t>Biology</t>
         </is>
       </c>
-      <c r="H7" s="12" t="inlineStr">
+      <c r="H7" s="13" t="inlineStr">
         <is>
           <t>Russian</t>
         </is>
@@ -1199,40 +1299,40 @@
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="11" t="n">
+      <c r="A9" s="12" t="n">
         <v>6</v>
       </c>
-      <c r="B9" s="12" t="inlineStr">
+      <c r="B9" s="13" t="inlineStr">
         <is>
           <t>Rashidov Ayyubxon</t>
         </is>
       </c>
-      <c r="C9" s="13" t="inlineStr">
+      <c r="C9" s="14" t="inlineStr">
         <is>
           <t>8-P</t>
         </is>
       </c>
-      <c r="D9" s="12" t="inlineStr">
-        <is>
-          <t>Mathematics</t>
-        </is>
-      </c>
-      <c r="E9" s="12" t="inlineStr">
+      <c r="D9" s="10" t="inlineStr">
+        <is>
+          <t>Mathematics</t>
+        </is>
+      </c>
+      <c r="E9" s="13" t="inlineStr">
         <is>
           <t>Physics</t>
         </is>
       </c>
-      <c r="F9" s="12" t="inlineStr">
+      <c r="F9" s="13" t="inlineStr">
         <is>
           <t>Chemistry</t>
         </is>
       </c>
-      <c r="G9" s="12" t="inlineStr">
-        <is>
-          <t>English</t>
-        </is>
-      </c>
-      <c r="H9" s="12" t="inlineStr">
+      <c r="G9" s="13" t="inlineStr">
+        <is>
+          <t>English</t>
+        </is>
+      </c>
+      <c r="H9" s="13" t="inlineStr">
         <is>
           <t>Uzbek / Russian</t>
         </is>
@@ -1257,7 +1357,7 @@
           <t>English</t>
         </is>
       </c>
-      <c r="E10" s="8" t="inlineStr">
+      <c r="E10" s="18" t="inlineStr">
         <is>
           <t>Biology</t>
         </is>
@@ -1279,40 +1379,40 @@
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="11" t="n">
+      <c r="A11" s="12" t="n">
         <v>8</v>
       </c>
-      <c r="B11" s="12" t="inlineStr">
+      <c r="B11" s="13" t="inlineStr">
         <is>
           <t>J. Umar</t>
         </is>
       </c>
-      <c r="C11" s="13" t="inlineStr">
+      <c r="C11" s="14" t="inlineStr">
         <is>
           <t>8-P</t>
         </is>
       </c>
-      <c r="D11" s="12" t="inlineStr">
-        <is>
-          <t>Mathematics</t>
-        </is>
-      </c>
-      <c r="E11" s="12" t="inlineStr">
+      <c r="D11" s="10" t="inlineStr">
+        <is>
+          <t>Mathematics</t>
+        </is>
+      </c>
+      <c r="E11" s="13" t="inlineStr">
         <is>
           <t>Robotics</t>
         </is>
       </c>
-      <c r="F11" s="12" t="inlineStr">
-        <is>
-          <t>English</t>
-        </is>
-      </c>
-      <c r="G11" s="12" t="inlineStr">
+      <c r="F11" s="13" t="inlineStr">
+        <is>
+          <t>English</t>
+        </is>
+      </c>
+      <c r="G11" s="13" t="inlineStr">
         <is>
           <t>Physics</t>
         </is>
       </c>
-      <c r="H11" s="12" t="inlineStr">
+      <c r="H11" s="13" t="inlineStr">
         <is>
           <t>IT</t>
         </is>
@@ -1347,7 +1447,7 @@
           <t>History</t>
         </is>
       </c>
-      <c r="G12" s="8" t="inlineStr">
+      <c r="G12" s="20" t="inlineStr">
         <is>
           <t>Chemistry</t>
         </is>
@@ -1359,36 +1459,36 @@
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="11" t="n">
+      <c r="A13" s="12" t="n">
         <v>10</v>
       </c>
-      <c r="B13" s="12" t="inlineStr">
+      <c r="B13" s="13" t="inlineStr">
         <is>
           <t>Shuhratov Johongir</t>
         </is>
       </c>
-      <c r="C13" s="13" t="inlineStr">
+      <c r="C13" s="14" t="inlineStr">
         <is>
           <t>8-A</t>
         </is>
       </c>
-      <c r="D13" s="12" t="inlineStr">
-        <is>
-          <t>Mathematics</t>
-        </is>
-      </c>
-      <c r="E13" s="12" t="inlineStr">
+      <c r="D13" s="13" t="inlineStr">
+        <is>
+          <t>Mathematics</t>
+        </is>
+      </c>
+      <c r="E13" s="15" t="inlineStr">
         <is>
           <t>Physics</t>
         </is>
       </c>
-      <c r="F13" s="12" t="inlineStr">
-        <is>
-          <t>English</t>
-        </is>
-      </c>
-      <c r="G13" s="14" t="n"/>
-      <c r="H13" s="14" t="n"/>
+      <c r="F13" s="13" t="inlineStr">
+        <is>
+          <t>English</t>
+        </is>
+      </c>
+      <c r="G13" s="17" t="n"/>
+      <c r="H13" s="17" t="n"/>
     </row>
     <row r="14">
       <c r="A14" s="7" t="n">
@@ -1404,7 +1504,7 @@
           <t>8-P</t>
         </is>
       </c>
-      <c r="D14" s="8" t="inlineStr">
+      <c r="D14" s="10" t="inlineStr">
         <is>
           <t>Mathematics</t>
         </is>
@@ -1431,40 +1531,40 @@
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="11" t="n">
+      <c r="A15" s="12" t="n">
         <v>12</v>
       </c>
-      <c r="B15" s="12" t="inlineStr">
+      <c r="B15" s="13" t="inlineStr">
         <is>
           <t>Muhammadali Kasimov</t>
         </is>
       </c>
-      <c r="C15" s="13" t="inlineStr">
+      <c r="C15" s="14" t="inlineStr">
         <is>
           <t>8-G</t>
         </is>
       </c>
-      <c r="D15" s="12" t="inlineStr">
-        <is>
-          <t>English</t>
-        </is>
-      </c>
-      <c r="E15" s="12" t="inlineStr">
+      <c r="D15" s="13" t="inlineStr">
+        <is>
+          <t>English</t>
+        </is>
+      </c>
+      <c r="E15" s="20" t="inlineStr">
         <is>
           <t>Chemistry</t>
         </is>
       </c>
-      <c r="F15" s="12" t="inlineStr">
-        <is>
-          <t>Mathematics</t>
-        </is>
-      </c>
-      <c r="G15" s="12" t="inlineStr">
+      <c r="F15" s="13" t="inlineStr">
+        <is>
+          <t>Mathematics</t>
+        </is>
+      </c>
+      <c r="G15" s="13" t="inlineStr">
         <is>
           <t>Geography</t>
         </is>
       </c>
-      <c r="H15" s="14" t="n"/>
+      <c r="H15" s="17" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="1">
@@ -1556,7 +1656,7 @@
           <t>9-G</t>
         </is>
       </c>
-      <c r="D4" s="8" t="inlineStr">
+      <c r="D4" s="10" t="inlineStr">
         <is>
           <t>Mathematics</t>
         </is>
@@ -1583,36 +1683,36 @@
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="11" t="n">
+      <c r="A5" s="12" t="n">
         <v>2</v>
       </c>
-      <c r="B5" s="12" t="inlineStr">
+      <c r="B5" s="13" t="inlineStr">
         <is>
           <t>Anvar Maksumov</t>
         </is>
       </c>
-      <c r="C5" s="13" t="inlineStr">
+      <c r="C5" s="14" t="inlineStr">
         <is>
           <t>9-B</t>
         </is>
       </c>
-      <c r="D5" s="12" t="inlineStr">
-        <is>
-          <t>Mathematics</t>
-        </is>
-      </c>
-      <c r="E5" s="12" t="inlineStr">
-        <is>
-          <t>English</t>
-        </is>
-      </c>
-      <c r="F5" s="12" t="inlineStr">
+      <c r="D5" s="10" t="inlineStr">
+        <is>
+          <t>Mathematics</t>
+        </is>
+      </c>
+      <c r="E5" s="13" t="inlineStr">
+        <is>
+          <t>English</t>
+        </is>
+      </c>
+      <c r="F5" s="13" t="inlineStr">
         <is>
           <t>Russian</t>
         </is>
       </c>
-      <c r="G5" s="14" t="n"/>
-      <c r="H5" s="14" t="n"/>
+      <c r="G5" s="17" t="n"/>
+      <c r="H5" s="17" t="n"/>
     </row>
     <row r="6">
       <c r="A6" s="7" t="n">
@@ -1628,7 +1728,7 @@
           <t>9-A</t>
         </is>
       </c>
-      <c r="D6" s="8" t="inlineStr">
+      <c r="D6" s="16" t="inlineStr">
         <is>
           <t>English</t>
         </is>
@@ -1655,40 +1755,40 @@
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="11" t="n">
+      <c r="A7" s="12" t="n">
         <v>4</v>
       </c>
-      <c r="B7" s="12" t="inlineStr">
+      <c r="B7" s="13" t="inlineStr">
         <is>
           <t>Murtazaeva Muzayyana</t>
         </is>
       </c>
-      <c r="C7" s="13" t="inlineStr">
+      <c r="C7" s="14" t="inlineStr">
         <is>
           <t>9-A</t>
         </is>
       </c>
-      <c r="D7" s="12" t="inlineStr">
-        <is>
-          <t>English</t>
-        </is>
-      </c>
-      <c r="E7" s="12" t="inlineStr">
+      <c r="D7" s="16" t="inlineStr">
+        <is>
+          <t>English</t>
+        </is>
+      </c>
+      <c r="E7" s="13" t="inlineStr">
         <is>
           <t>Geography</t>
         </is>
       </c>
-      <c r="F7" s="12" t="inlineStr">
+      <c r="F7" s="13" t="inlineStr">
         <is>
           <t>History</t>
         </is>
       </c>
-      <c r="G7" s="12" t="inlineStr">
-        <is>
-          <t>Mathematics</t>
-        </is>
-      </c>
-      <c r="H7" s="14" t="n"/>
+      <c r="G7" s="13" t="inlineStr">
+        <is>
+          <t>Mathematics</t>
+        </is>
+      </c>
+      <c r="H7" s="17" t="n"/>
     </row>
     <row r="8">
       <c r="A8" s="7" t="n">
@@ -1714,7 +1814,7 @@
           <t>Physics</t>
         </is>
       </c>
-      <c r="F8" s="8" t="inlineStr">
+      <c r="F8" s="19" t="inlineStr">
         <is>
           <t>History</t>
         </is>
@@ -1724,39 +1824,39 @@
           <t>Geography</t>
         </is>
       </c>
-      <c r="H8" s="10" t="n"/>
+      <c r="H8" s="11" t="n"/>
     </row>
     <row r="9">
-      <c r="A9" s="11" t="n">
+      <c r="A9" s="12" t="n">
         <v>6</v>
       </c>
-      <c r="B9" s="12" t="inlineStr">
+      <c r="B9" s="13" t="inlineStr">
         <is>
           <t>Parviz</t>
         </is>
       </c>
-      <c r="C9" s="13" t="inlineStr">
+      <c r="C9" s="14" t="inlineStr">
         <is>
           <t>9-A</t>
         </is>
       </c>
-      <c r="D9" s="12" t="inlineStr">
-        <is>
-          <t>English</t>
-        </is>
-      </c>
-      <c r="E9" s="12" t="inlineStr">
-        <is>
-          <t>Mathematics</t>
-        </is>
-      </c>
-      <c r="F9" s="12" t="inlineStr">
+      <c r="D9" s="13" t="inlineStr">
+        <is>
+          <t>English</t>
+        </is>
+      </c>
+      <c r="E9" s="13" t="inlineStr">
+        <is>
+          <t>Mathematics</t>
+        </is>
+      </c>
+      <c r="F9" s="21" t="inlineStr">
         <is>
           <t>IT</t>
         </is>
       </c>
-      <c r="G9" s="14" t="n"/>
-      <c r="H9" s="14" t="n"/>
+      <c r="G9" s="17" t="n"/>
+      <c r="H9" s="17" t="n"/>
     </row>
     <row r="10">
       <c r="A10" s="7" t="n">
@@ -1772,7 +1872,7 @@
           <t>9-A</t>
         </is>
       </c>
-      <c r="D10" s="8" t="inlineStr">
+      <c r="D10" s="21" t="inlineStr">
         <is>
           <t>IT</t>
         </is>
@@ -1787,44 +1887,44 @@
           <t>Biology</t>
         </is>
       </c>
-      <c r="G10" s="10" t="n"/>
-      <c r="H10" s="10" t="n"/>
+      <c r="G10" s="11" t="n"/>
+      <c r="H10" s="11" t="n"/>
     </row>
     <row r="11">
-      <c r="A11" s="11" t="n">
+      <c r="A11" s="12" t="n">
         <v>8</v>
       </c>
-      <c r="B11" s="12" t="inlineStr">
+      <c r="B11" s="13" t="inlineStr">
         <is>
           <t>Tojiddinova Hadicha</t>
         </is>
       </c>
-      <c r="C11" s="13" t="inlineStr">
+      <c r="C11" s="14" t="inlineStr">
         <is>
           <t>9-G</t>
         </is>
       </c>
-      <c r="D11" s="12" t="inlineStr">
-        <is>
-          <t>Mathematics</t>
-        </is>
-      </c>
-      <c r="E11" s="12" t="inlineStr">
-        <is>
-          <t>English</t>
-        </is>
-      </c>
-      <c r="F11" s="12" t="inlineStr">
+      <c r="D11" s="10" t="inlineStr">
+        <is>
+          <t>Mathematics</t>
+        </is>
+      </c>
+      <c r="E11" s="13" t="inlineStr">
+        <is>
+          <t>English</t>
+        </is>
+      </c>
+      <c r="F11" s="13" t="inlineStr">
         <is>
           <t>History</t>
         </is>
       </c>
-      <c r="G11" s="12" t="inlineStr">
+      <c r="G11" s="13" t="inlineStr">
         <is>
           <t>Geography</t>
         </is>
       </c>
-      <c r="H11" s="12" t="inlineStr">
+      <c r="H11" s="13" t="inlineStr">
         <is>
           <t>Physics</t>
         </is>
@@ -1844,7 +1944,7 @@
           <t>9</t>
         </is>
       </c>
-      <c r="D12" s="8" t="inlineStr">
+      <c r="D12" s="18" t="inlineStr">
         <is>
           <t>Biology</t>
         </is>
@@ -1960,7 +2060,7 @@
           <t>10-A</t>
         </is>
       </c>
-      <c r="D4" s="8" t="inlineStr">
+      <c r="D4" s="15" t="inlineStr">
         <is>
           <t>Physics</t>
         </is>
@@ -1975,36 +2075,36 @@
           <t>English</t>
         </is>
       </c>
-      <c r="G4" s="10" t="n"/>
-      <c r="H4" s="10" t="n"/>
+      <c r="G4" s="11" t="n"/>
+      <c r="H4" s="11" t="n"/>
     </row>
     <row r="5">
-      <c r="A5" s="11" t="n">
+      <c r="A5" s="12" t="n">
         <v>2</v>
       </c>
-      <c r="B5" s="12" t="inlineStr">
+      <c r="B5" s="13" t="inlineStr">
         <is>
           <t>Islomov Xondamir</t>
         </is>
       </c>
-      <c r="C5" s="13" t="inlineStr">
+      <c r="C5" s="14" t="inlineStr">
         <is>
           <t>10-A</t>
         </is>
       </c>
-      <c r="D5" s="12" t="inlineStr">
+      <c r="D5" s="13" t="inlineStr">
         <is>
           <t>Law</t>
         </is>
       </c>
-      <c r="E5" s="12" t="inlineStr">
+      <c r="E5" s="13" t="inlineStr">
         <is>
           <t>National Defense (OZI)</t>
         </is>
       </c>
-      <c r="F5" s="14" t="n"/>
-      <c r="G5" s="14" t="n"/>
-      <c r="H5" s="14" t="n"/>
+      <c r="F5" s="17" t="n"/>
+      <c r="G5" s="17" t="n"/>
+      <c r="H5" s="17" t="n"/>
     </row>
     <row r="6">
       <c r="A6" s="7" t="n">
@@ -2020,7 +2120,7 @@
           <t>10-A</t>
         </is>
       </c>
-      <c r="D6" s="8" t="inlineStr">
+      <c r="D6" s="10" t="inlineStr">
         <is>
           <t>Mathematics</t>
         </is>
@@ -2035,44 +2135,44 @@
           <t>English</t>
         </is>
       </c>
-      <c r="G6" s="10" t="n"/>
-      <c r="H6" s="10" t="n"/>
+      <c r="G6" s="11" t="n"/>
+      <c r="H6" s="11" t="n"/>
     </row>
     <row r="7">
-      <c r="A7" s="11" t="n">
+      <c r="A7" s="12" t="n">
         <v>4</v>
       </c>
-      <c r="B7" s="12" t="inlineStr">
+      <c r="B7" s="13" t="inlineStr">
         <is>
           <t>Baxtiyorov Biloliddin</t>
         </is>
       </c>
-      <c r="C7" s="13" t="inlineStr">
+      <c r="C7" s="14" t="inlineStr">
         <is>
           <t>10</t>
         </is>
       </c>
-      <c r="D7" s="12" t="inlineStr">
-        <is>
-          <t>English</t>
-        </is>
-      </c>
-      <c r="E7" s="12" t="inlineStr">
-        <is>
-          <t>Mathematics</t>
-        </is>
-      </c>
-      <c r="F7" s="12" t="inlineStr">
+      <c r="D7" s="16" t="inlineStr">
+        <is>
+          <t>English</t>
+        </is>
+      </c>
+      <c r="E7" s="13" t="inlineStr">
+        <is>
+          <t>Mathematics</t>
+        </is>
+      </c>
+      <c r="F7" s="13" t="inlineStr">
         <is>
           <t>Physics</t>
         </is>
       </c>
-      <c r="G7" s="12" t="inlineStr">
+      <c r="G7" s="13" t="inlineStr">
         <is>
           <t>ICT</t>
         </is>
       </c>
-      <c r="H7" s="14" t="n"/>
+      <c r="H7" s="17" t="n"/>
     </row>
     <row r="8">
       <c r="A8" s="7" t="n">
@@ -2088,51 +2188,51 @@
           <t>10-G</t>
         </is>
       </c>
-      <c r="D8" s="8" t="inlineStr">
-        <is>
-          <t>Mathematics</t>
-        </is>
-      </c>
-      <c r="E8" s="10" t="n"/>
-      <c r="F8" s="10" t="n"/>
-      <c r="G8" s="10" t="n"/>
-      <c r="H8" s="10" t="n"/>
+      <c r="D8" s="10" t="inlineStr">
+        <is>
+          <t>Mathematics</t>
+        </is>
+      </c>
+      <c r="E8" s="11" t="n"/>
+      <c r="F8" s="11" t="n"/>
+      <c r="G8" s="11" t="n"/>
+      <c r="H8" s="11" t="n"/>
     </row>
     <row r="9">
-      <c r="A9" s="11" t="n">
+      <c r="A9" s="12" t="n">
         <v>6</v>
       </c>
-      <c r="B9" s="12" t="inlineStr">
+      <c r="B9" s="13" t="inlineStr">
         <is>
           <t>Xudoynazarova Nodira</t>
         </is>
       </c>
-      <c r="C9" s="13" t="inlineStr">
+      <c r="C9" s="14" t="inlineStr">
         <is>
           <t>10-B</t>
         </is>
       </c>
-      <c r="D9" s="12" t="inlineStr">
+      <c r="D9" s="21" t="inlineStr">
         <is>
           <t>IT</t>
         </is>
       </c>
-      <c r="E9" s="12" t="inlineStr">
-        <is>
-          <t>Mathematics</t>
-        </is>
-      </c>
-      <c r="F9" s="12" t="inlineStr">
+      <c r="E9" s="13" t="inlineStr">
+        <is>
+          <t>Mathematics</t>
+        </is>
+      </c>
+      <c r="F9" s="13" t="inlineStr">
         <is>
           <t>Physics</t>
         </is>
       </c>
-      <c r="G9" s="12" t="inlineStr">
+      <c r="G9" s="13" t="inlineStr">
         <is>
           <t>Biology</t>
         </is>
       </c>
-      <c r="H9" s="14" t="n"/>
+      <c r="H9" s="17" t="n"/>
     </row>
     <row r="10">
       <c r="A10" s="7" t="n">
@@ -2148,7 +2248,7 @@
           <t>10</t>
         </is>
       </c>
-      <c r="D10" s="8" t="inlineStr">
+      <c r="D10" s="16" t="inlineStr">
         <is>
           <t>English</t>
         </is>
@@ -2168,7 +2268,7 @@
           <t>Biology</t>
         </is>
       </c>
-      <c r="H10" s="10" t="n"/>
+      <c r="H10" s="11" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="1">
@@ -2252,7 +2352,7 @@
       </c>
       <c r="B4" s="8" t="inlineStr">
         <is>
-          <t>Shukurullaeva Madinobonu</t>
+          <t>Shukurullaeva Madinabonu</t>
         </is>
       </c>
       <c r="C4" s="9" t="inlineStr">
@@ -2260,7 +2360,7 @@
           <t>11-A</t>
         </is>
       </c>
-      <c r="D4" s="8" t="inlineStr">
+      <c r="D4" s="16" t="inlineStr">
         <is>
           <t>English</t>
         </is>
@@ -2287,36 +2387,36 @@
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="11" t="n">
+      <c r="A5" s="12" t="n">
         <v>2</v>
       </c>
-      <c r="B5" s="12" t="inlineStr">
+      <c r="B5" s="13" t="inlineStr">
         <is>
           <t>Karimova Shahina</t>
         </is>
       </c>
-      <c r="C5" s="13" t="inlineStr">
+      <c r="C5" s="14" t="inlineStr">
         <is>
           <t>11-G</t>
         </is>
       </c>
-      <c r="D5" s="12" t="inlineStr">
-        <is>
-          <t>Mathematics</t>
-        </is>
-      </c>
-      <c r="E5" s="12" t="inlineStr">
+      <c r="D5" s="10" t="inlineStr">
+        <is>
+          <t>Mathematics</t>
+        </is>
+      </c>
+      <c r="E5" s="13" t="inlineStr">
         <is>
           <t>Native Language</t>
         </is>
       </c>
-      <c r="F5" s="12" t="inlineStr">
+      <c r="F5" s="13" t="inlineStr">
         <is>
           <t>Physical Education</t>
         </is>
       </c>
-      <c r="G5" s="14" t="n"/>
-      <c r="H5" s="14" t="n"/>
+      <c r="G5" s="17" t="n"/>
+      <c r="H5" s="17" t="n"/>
     </row>
     <row r="6">
       <c r="A6" s="7" t="n">
@@ -2332,7 +2432,7 @@
           <t>11-A</t>
         </is>
       </c>
-      <c r="D6" s="8" t="inlineStr">
+      <c r="D6" s="16" t="inlineStr">
         <is>
           <t>English</t>
         </is>
@@ -2359,40 +2459,40 @@
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="11" t="n">
+      <c r="A7" s="12" t="n">
         <v>4</v>
       </c>
-      <c r="B7" s="12" t="inlineStr">
+      <c r="B7" s="13" t="inlineStr">
         <is>
           <t>Solihabonu</t>
         </is>
       </c>
-      <c r="C7" s="13" t="inlineStr">
+      <c r="C7" s="14" t="inlineStr">
         <is>
           <t>11-G</t>
         </is>
       </c>
-      <c r="D7" s="12" t="inlineStr">
-        <is>
-          <t>Mathematics</t>
-        </is>
-      </c>
-      <c r="E7" s="12" t="inlineStr">
+      <c r="D7" s="10" t="inlineStr">
+        <is>
+          <t>Mathematics</t>
+        </is>
+      </c>
+      <c r="E7" s="13" t="inlineStr">
         <is>
           <t>Native Language (Uzbek)</t>
         </is>
       </c>
-      <c r="F7" s="12" t="inlineStr">
-        <is>
-          <t>English</t>
-        </is>
-      </c>
-      <c r="G7" s="12" t="inlineStr">
+      <c r="F7" s="13" t="inlineStr">
+        <is>
+          <t>English</t>
+        </is>
+      </c>
+      <c r="G7" s="13" t="inlineStr">
         <is>
           <t>History</t>
         </is>
       </c>
-      <c r="H7" s="12" t="inlineStr">
+      <c r="H7" s="13" t="inlineStr">
         <is>
           <t>ICT</t>
         </is>
@@ -2412,51 +2512,51 @@
           <t>11-G</t>
         </is>
       </c>
-      <c r="D8" s="8" t="inlineStr">
-        <is>
-          <t>English</t>
-        </is>
-      </c>
-      <c r="E8" s="10" t="n"/>
-      <c r="F8" s="10" t="n"/>
-      <c r="G8" s="10" t="n"/>
-      <c r="H8" s="10" t="n"/>
+      <c r="D8" s="16" t="inlineStr">
+        <is>
+          <t>English</t>
+        </is>
+      </c>
+      <c r="E8" s="11" t="n"/>
+      <c r="F8" s="11" t="n"/>
+      <c r="G8" s="11" t="n"/>
+      <c r="H8" s="11" t="n"/>
     </row>
     <row r="9">
-      <c r="A9" s="11" t="n">
+      <c r="A9" s="12" t="n">
         <v>6</v>
       </c>
-      <c r="B9" s="12" t="inlineStr">
+      <c r="B9" s="13" t="inlineStr">
         <is>
           <t>Shohjahon Qahhorov</t>
         </is>
       </c>
-      <c r="C9" s="13" t="inlineStr">
+      <c r="C9" s="14" t="inlineStr">
         <is>
           <t>11-G</t>
         </is>
       </c>
-      <c r="D9" s="12" t="inlineStr">
-        <is>
-          <t>English</t>
-        </is>
-      </c>
-      <c r="E9" s="12" t="inlineStr">
+      <c r="D9" s="13" t="inlineStr">
+        <is>
+          <t>English</t>
+        </is>
+      </c>
+      <c r="E9" s="15" t="inlineStr">
         <is>
           <t>Physics</t>
         </is>
       </c>
-      <c r="F9" s="12" t="inlineStr">
-        <is>
-          <t>Mathematics</t>
-        </is>
-      </c>
-      <c r="G9" s="12" t="inlineStr">
+      <c r="F9" s="13" t="inlineStr">
+        <is>
+          <t>Mathematics</t>
+        </is>
+      </c>
+      <c r="G9" s="13" t="inlineStr">
         <is>
           <t>Chemistry</t>
         </is>
       </c>
-      <c r="H9" s="14" t="n"/>
+      <c r="H9" s="17" t="n"/>
     </row>
     <row r="10">
       <c r="A10" s="7" t="n">
@@ -2477,7 +2577,7 @@
           <t>Mathematics</t>
         </is>
       </c>
-      <c r="E10" s="8" t="inlineStr">
+      <c r="E10" s="15" t="inlineStr">
         <is>
           <t>Physics</t>
         </is>
@@ -2504,4 +2604,1248 @@
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:E72"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="5" customWidth="1" min="1" max="1"/>
+    <col width="32" customWidth="1" min="2" max="2"/>
+    <col width="10" customWidth="1" min="3" max="3"/>
+    <col width="10" customWidth="1" min="4" max="4"/>
+    <col width="22" customWidth="1" min="5" max="5"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Ellipse International School - Students by Selected Olympiad Subject</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="2" t="inlineStr">
+        <is>
+          <t>#</t>
+        </is>
+      </c>
+      <c r="B3" s="2" t="inlineStr">
+        <is>
+          <t>Student Name</t>
+        </is>
+      </c>
+      <c r="C3" s="2" t="inlineStr">
+        <is>
+          <t>Class</t>
+        </is>
+      </c>
+      <c r="D3" s="2" t="inlineStr">
+        <is>
+          <t>Grade</t>
+        </is>
+      </c>
+      <c r="E3" s="2" t="inlineStr">
+        <is>
+          <t>Selected Subject</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="22" t="inlineStr">
+        <is>
+          <t>Mathematics (15 students)</t>
+        </is>
+      </c>
+      <c r="B4" s="11" t="n"/>
+      <c r="C4" s="11" t="n"/>
+      <c r="D4" s="11" t="n"/>
+      <c r="E4" s="11" t="n"/>
+    </row>
+    <row r="5">
+      <c r="A5" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="B5" s="8" t="inlineStr">
+        <is>
+          <t>Abdurasulov Abdulaziz</t>
+        </is>
+      </c>
+      <c r="C5" s="9" t="inlineStr">
+        <is>
+          <t>7-P</t>
+        </is>
+      </c>
+      <c r="D5" s="3" t="n">
+        <v>7</v>
+      </c>
+      <c r="E5" s="10" t="inlineStr">
+        <is>
+          <t>Mathematics</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="12" t="n">
+        <v>2</v>
+      </c>
+      <c r="B6" s="13" t="inlineStr">
+        <is>
+          <t>Dexkanova Bibixonim</t>
+        </is>
+      </c>
+      <c r="C6" s="14" t="inlineStr">
+        <is>
+          <t>7-P</t>
+        </is>
+      </c>
+      <c r="D6" s="4" t="n">
+        <v>7</v>
+      </c>
+      <c r="E6" s="10" t="inlineStr">
+        <is>
+          <t>Mathematics</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="7" t="n">
+        <v>3</v>
+      </c>
+      <c r="B7" s="8" t="inlineStr">
+        <is>
+          <t>Kulboeva Medina-Aisha</t>
+        </is>
+      </c>
+      <c r="C7" s="9" t="inlineStr">
+        <is>
+          <t>7-P</t>
+        </is>
+      </c>
+      <c r="D7" s="3" t="n">
+        <v>7</v>
+      </c>
+      <c r="E7" s="10" t="inlineStr">
+        <is>
+          <t>Mathematics</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="12" t="n">
+        <v>4</v>
+      </c>
+      <c r="B8" s="13" t="inlineStr">
+        <is>
+          <t>Ziyo</t>
+        </is>
+      </c>
+      <c r="C8" s="14" t="inlineStr">
+        <is>
+          <t>7-A</t>
+        </is>
+      </c>
+      <c r="D8" s="4" t="n">
+        <v>7</v>
+      </c>
+      <c r="E8" s="10" t="inlineStr">
+        <is>
+          <t>Mathematics</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="7" t="n">
+        <v>5</v>
+      </c>
+      <c r="B9" s="8" t="inlineStr">
+        <is>
+          <t>Baxtiyorov Imron</t>
+        </is>
+      </c>
+      <c r="C9" s="9" t="inlineStr">
+        <is>
+          <t>8-P</t>
+        </is>
+      </c>
+      <c r="D9" s="3" t="n">
+        <v>8</v>
+      </c>
+      <c r="E9" s="10" t="inlineStr">
+        <is>
+          <t>Mathematics</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="12" t="n">
+        <v>6</v>
+      </c>
+      <c r="B10" s="13" t="inlineStr">
+        <is>
+          <t>J. Umar</t>
+        </is>
+      </c>
+      <c r="C10" s="14" t="inlineStr">
+        <is>
+          <t>8-P</t>
+        </is>
+      </c>
+      <c r="D10" s="4" t="n">
+        <v>8</v>
+      </c>
+      <c r="E10" s="10" t="inlineStr">
+        <is>
+          <t>Mathematics</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="7" t="n">
+        <v>7</v>
+      </c>
+      <c r="B11" s="8" t="inlineStr">
+        <is>
+          <t>Rashidov Ayyubxon</t>
+        </is>
+      </c>
+      <c r="C11" s="9" t="inlineStr">
+        <is>
+          <t>8-P</t>
+        </is>
+      </c>
+      <c r="D11" s="3" t="n">
+        <v>8</v>
+      </c>
+      <c r="E11" s="10" t="inlineStr">
+        <is>
+          <t>Mathematics</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="12" t="n">
+        <v>8</v>
+      </c>
+      <c r="B12" s="13" t="inlineStr">
+        <is>
+          <t>Xasanova Latofat</t>
+        </is>
+      </c>
+      <c r="C12" s="14" t="inlineStr">
+        <is>
+          <t>8-P</t>
+        </is>
+      </c>
+      <c r="D12" s="4" t="n">
+        <v>8</v>
+      </c>
+      <c r="E12" s="10" t="inlineStr">
+        <is>
+          <t>Mathematics</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="7" t="n">
+        <v>9</v>
+      </c>
+      <c r="B13" s="8" t="inlineStr">
+        <is>
+          <t>Anvar Maksumov</t>
+        </is>
+      </c>
+      <c r="C13" s="9" t="inlineStr">
+        <is>
+          <t>9-B</t>
+        </is>
+      </c>
+      <c r="D13" s="3" t="n">
+        <v>9</v>
+      </c>
+      <c r="E13" s="10" t="inlineStr">
+        <is>
+          <t>Mathematics</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="12" t="n">
+        <v>10</v>
+      </c>
+      <c r="B14" s="13" t="inlineStr">
+        <is>
+          <t>Ismoilov Otabek</t>
+        </is>
+      </c>
+      <c r="C14" s="14" t="inlineStr">
+        <is>
+          <t>9-G</t>
+        </is>
+      </c>
+      <c r="D14" s="4" t="n">
+        <v>9</v>
+      </c>
+      <c r="E14" s="10" t="inlineStr">
+        <is>
+          <t>Mathematics</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="7" t="n">
+        <v>11</v>
+      </c>
+      <c r="B15" s="8" t="inlineStr">
+        <is>
+          <t>Tojiddinova Hadicha</t>
+        </is>
+      </c>
+      <c r="C15" s="9" t="inlineStr">
+        <is>
+          <t>9-G</t>
+        </is>
+      </c>
+      <c r="D15" s="3" t="n">
+        <v>9</v>
+      </c>
+      <c r="E15" s="10" t="inlineStr">
+        <is>
+          <t>Mathematics</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="12" t="n">
+        <v>12</v>
+      </c>
+      <c r="B16" s="13" t="inlineStr">
+        <is>
+          <t>Sulaimon Saidakbar</t>
+        </is>
+      </c>
+      <c r="C16" s="14" t="inlineStr">
+        <is>
+          <t>10-A</t>
+        </is>
+      </c>
+      <c r="D16" s="4" t="n">
+        <v>10</v>
+      </c>
+      <c r="E16" s="10" t="inlineStr">
+        <is>
+          <t>Mathematics</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="7" t="n">
+        <v>13</v>
+      </c>
+      <c r="B17" s="8" t="inlineStr">
+        <is>
+          <t>Turaev Sardor</t>
+        </is>
+      </c>
+      <c r="C17" s="9" t="inlineStr">
+        <is>
+          <t>10-G</t>
+        </is>
+      </c>
+      <c r="D17" s="3" t="n">
+        <v>10</v>
+      </c>
+      <c r="E17" s="10" t="inlineStr">
+        <is>
+          <t>Mathematics</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="12" t="n">
+        <v>14</v>
+      </c>
+      <c r="B18" s="13" t="inlineStr">
+        <is>
+          <t>Karimova Shahina</t>
+        </is>
+      </c>
+      <c r="C18" s="14" t="inlineStr">
+        <is>
+          <t>11-G</t>
+        </is>
+      </c>
+      <c r="D18" s="4" t="n">
+        <v>11</v>
+      </c>
+      <c r="E18" s="10" t="inlineStr">
+        <is>
+          <t>Mathematics</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="7" t="n">
+        <v>15</v>
+      </c>
+      <c r="B19" s="8" t="inlineStr">
+        <is>
+          <t>Solihabonu</t>
+        </is>
+      </c>
+      <c r="C19" s="9" t="inlineStr">
+        <is>
+          <t>11-G</t>
+        </is>
+      </c>
+      <c r="D19" s="3" t="n">
+        <v>11</v>
+      </c>
+      <c r="E19" s="10" t="inlineStr">
+        <is>
+          <t>Mathematics</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="23" t="inlineStr">
+        <is>
+          <t>Physics (6 students)</t>
+        </is>
+      </c>
+      <c r="B21" s="11" t="n"/>
+      <c r="C21" s="11" t="n"/>
+      <c r="D21" s="11" t="n"/>
+      <c r="E21" s="11" t="n"/>
+    </row>
+    <row r="22">
+      <c r="A22" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="B22" s="8" t="inlineStr">
+        <is>
+          <t>Avazbek Mirzaazizov</t>
+        </is>
+      </c>
+      <c r="C22" s="9" t="inlineStr">
+        <is>
+          <t>7-A</t>
+        </is>
+      </c>
+      <c r="D22" s="3" t="n">
+        <v>7</v>
+      </c>
+      <c r="E22" s="15" t="inlineStr">
+        <is>
+          <t>Physics</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="12" t="n">
+        <v>2</v>
+      </c>
+      <c r="B23" s="13" t="inlineStr">
+        <is>
+          <t>Muhammad Yosin</t>
+        </is>
+      </c>
+      <c r="C23" s="14" t="inlineStr">
+        <is>
+          <t>7-P</t>
+        </is>
+      </c>
+      <c r="D23" s="4" t="n">
+        <v>7</v>
+      </c>
+      <c r="E23" s="15" t="inlineStr">
+        <is>
+          <t>Physics</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="7" t="n">
+        <v>3</v>
+      </c>
+      <c r="B24" s="8" t="inlineStr">
+        <is>
+          <t>Shuhratov Johongir</t>
+        </is>
+      </c>
+      <c r="C24" s="9" t="inlineStr">
+        <is>
+          <t>8-A</t>
+        </is>
+      </c>
+      <c r="D24" s="3" t="n">
+        <v>8</v>
+      </c>
+      <c r="E24" s="15" t="inlineStr">
+        <is>
+          <t>Physics</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="12" t="n">
+        <v>4</v>
+      </c>
+      <c r="B25" s="13" t="inlineStr">
+        <is>
+          <t>Baboxodjaev Abdulla</t>
+        </is>
+      </c>
+      <c r="C25" s="14" t="inlineStr">
+        <is>
+          <t>10-A</t>
+        </is>
+      </c>
+      <c r="D25" s="4" t="n">
+        <v>10</v>
+      </c>
+      <c r="E25" s="15" t="inlineStr">
+        <is>
+          <t>Physics</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="7" t="n">
+        <v>5</v>
+      </c>
+      <c r="B26" s="8" t="inlineStr">
+        <is>
+          <t>Baxodirov Usmon</t>
+        </is>
+      </c>
+      <c r="C26" s="9" t="inlineStr">
+        <is>
+          <t>11-A</t>
+        </is>
+      </c>
+      <c r="D26" s="3" t="n">
+        <v>11</v>
+      </c>
+      <c r="E26" s="15" t="inlineStr">
+        <is>
+          <t>Physics</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="12" t="n">
+        <v>6</v>
+      </c>
+      <c r="B27" s="13" t="inlineStr">
+        <is>
+          <t>Shohjahon Qahhorov</t>
+        </is>
+      </c>
+      <c r="C27" s="14" t="inlineStr">
+        <is>
+          <t>11-G</t>
+        </is>
+      </c>
+      <c r="D27" s="4" t="n">
+        <v>11</v>
+      </c>
+      <c r="E27" s="15" t="inlineStr">
+        <is>
+          <t>Physics</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="24" t="inlineStr">
+        <is>
+          <t>English (8 students)</t>
+        </is>
+      </c>
+      <c r="B29" s="11" t="n"/>
+      <c r="C29" s="11" t="n"/>
+      <c r="D29" s="11" t="n"/>
+      <c r="E29" s="11" t="n"/>
+    </row>
+    <row r="30">
+      <c r="A30" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="B30" s="8" t="inlineStr">
+        <is>
+          <t>Uzakbaev Imon</t>
+        </is>
+      </c>
+      <c r="C30" s="9" t="inlineStr">
+        <is>
+          <t>7-B</t>
+        </is>
+      </c>
+      <c r="D30" s="3" t="n">
+        <v>7</v>
+      </c>
+      <c r="E30" s="16" t="inlineStr">
+        <is>
+          <t>English</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="12" t="n">
+        <v>2</v>
+      </c>
+      <c r="B31" s="13" t="inlineStr">
+        <is>
+          <t>Mirkobilova Rayyona</t>
+        </is>
+      </c>
+      <c r="C31" s="14" t="inlineStr">
+        <is>
+          <t>9-A</t>
+        </is>
+      </c>
+      <c r="D31" s="4" t="n">
+        <v>9</v>
+      </c>
+      <c r="E31" s="16" t="inlineStr">
+        <is>
+          <t>English</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="7" t="n">
+        <v>3</v>
+      </c>
+      <c r="B32" s="8" t="inlineStr">
+        <is>
+          <t>Murtazaeva Muzayyana</t>
+        </is>
+      </c>
+      <c r="C32" s="9" t="inlineStr">
+        <is>
+          <t>9-A</t>
+        </is>
+      </c>
+      <c r="D32" s="3" t="n">
+        <v>9</v>
+      </c>
+      <c r="E32" s="16" t="inlineStr">
+        <is>
+          <t>English</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="12" t="n">
+        <v>4</v>
+      </c>
+      <c r="B33" s="13" t="inlineStr">
+        <is>
+          <t>Baxtiyorov Biloliddin</t>
+        </is>
+      </c>
+      <c r="C33" s="14" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
+      </c>
+      <c r="D33" s="4" t="n">
+        <v>10</v>
+      </c>
+      <c r="E33" s="16" t="inlineStr">
+        <is>
+          <t>English</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="7" t="n">
+        <v>5</v>
+      </c>
+      <c r="B34" s="8" t="inlineStr">
+        <is>
+          <t>Kurbonalieva Madina</t>
+        </is>
+      </c>
+      <c r="C34" s="9" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
+      </c>
+      <c r="D34" s="3" t="n">
+        <v>10</v>
+      </c>
+      <c r="E34" s="16" t="inlineStr">
+        <is>
+          <t>English</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="12" t="n">
+        <v>6</v>
+      </c>
+      <c r="B35" s="13" t="inlineStr">
+        <is>
+          <t>Abdulxajieva Zaxro</t>
+        </is>
+      </c>
+      <c r="C35" s="14" t="inlineStr">
+        <is>
+          <t>11-A</t>
+        </is>
+      </c>
+      <c r="D35" s="4" t="n">
+        <v>11</v>
+      </c>
+      <c r="E35" s="16" t="inlineStr">
+        <is>
+          <t>English</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="7" t="n">
+        <v>7</v>
+      </c>
+      <c r="B36" s="8" t="inlineStr">
+        <is>
+          <t>Anvarxonov Saidalo</t>
+        </is>
+      </c>
+      <c r="C36" s="9" t="inlineStr">
+        <is>
+          <t>11-G</t>
+        </is>
+      </c>
+      <c r="D36" s="3" t="n">
+        <v>11</v>
+      </c>
+      <c r="E36" s="16" t="inlineStr">
+        <is>
+          <t>English</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="12" t="n">
+        <v>8</v>
+      </c>
+      <c r="B37" s="13" t="inlineStr">
+        <is>
+          <t>Shukurullaeva Madinabonu</t>
+        </is>
+      </c>
+      <c r="C37" s="14" t="inlineStr">
+        <is>
+          <t>11-A</t>
+        </is>
+      </c>
+      <c r="D37" s="4" t="n">
+        <v>11</v>
+      </c>
+      <c r="E37" s="16" t="inlineStr">
+        <is>
+          <t>English</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="25" t="inlineStr">
+        <is>
+          <t>Biology (4 students)</t>
+        </is>
+      </c>
+      <c r="B39" s="11" t="n"/>
+      <c r="C39" s="11" t="n"/>
+      <c r="D39" s="11" t="n"/>
+      <c r="E39" s="11" t="n"/>
+    </row>
+    <row r="40">
+      <c r="A40" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="B40" s="8" t="inlineStr">
+        <is>
+          <t>Abdujabborov Behruz</t>
+        </is>
+      </c>
+      <c r="C40" s="9" t="inlineStr">
+        <is>
+          <t>8-P</t>
+        </is>
+      </c>
+      <c r="D40" s="3" t="n">
+        <v>8</v>
+      </c>
+      <c r="E40" s="18" t="inlineStr">
+        <is>
+          <t>Biology</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="12" t="n">
+        <v>2</v>
+      </c>
+      <c r="B41" s="13" t="inlineStr">
+        <is>
+          <t>Boborova Gavxor</t>
+        </is>
+      </c>
+      <c r="C41" s="14" t="inlineStr">
+        <is>
+          <t>8-B</t>
+        </is>
+      </c>
+      <c r="D41" s="4" t="n">
+        <v>8</v>
+      </c>
+      <c r="E41" s="18" t="inlineStr">
+        <is>
+          <t>Biology</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="7" t="n">
+        <v>3</v>
+      </c>
+      <c r="B42" s="8" t="inlineStr">
+        <is>
+          <t>Muhammad Sanan</t>
+        </is>
+      </c>
+      <c r="C42" s="9" t="inlineStr">
+        <is>
+          <t>8-P</t>
+        </is>
+      </c>
+      <c r="D42" s="3" t="n">
+        <v>8</v>
+      </c>
+      <c r="E42" s="18" t="inlineStr">
+        <is>
+          <t>Biology</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="12" t="n">
+        <v>4</v>
+      </c>
+      <c r="B43" s="13" t="inlineStr">
+        <is>
+          <t>Abdusamadov Javokhir</t>
+        </is>
+      </c>
+      <c r="C43" s="14" t="inlineStr">
+        <is>
+          <t>9</t>
+        </is>
+      </c>
+      <c r="D43" s="4" t="n">
+        <v>9</v>
+      </c>
+      <c r="E43" s="18" t="inlineStr">
+        <is>
+          <t>Biology</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="26" t="inlineStr">
+        <is>
+          <t>Chemistry (2 students)</t>
+        </is>
+      </c>
+      <c r="B45" s="11" t="n"/>
+      <c r="C45" s="11" t="n"/>
+      <c r="D45" s="11" t="n"/>
+      <c r="E45" s="11" t="n"/>
+    </row>
+    <row r="46">
+      <c r="A46" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="B46" s="8" t="inlineStr">
+        <is>
+          <t>Ismailov Yusufxon</t>
+        </is>
+      </c>
+      <c r="C46" s="9" t="inlineStr">
+        <is>
+          <t>8-G</t>
+        </is>
+      </c>
+      <c r="D46" s="3" t="n">
+        <v>8</v>
+      </c>
+      <c r="E46" s="20" t="inlineStr">
+        <is>
+          <t>Chemistry</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="12" t="n">
+        <v>2</v>
+      </c>
+      <c r="B47" s="13" t="inlineStr">
+        <is>
+          <t>Muhammadali Kasimov</t>
+        </is>
+      </c>
+      <c r="C47" s="14" t="inlineStr">
+        <is>
+          <t>8-G</t>
+        </is>
+      </c>
+      <c r="D47" s="4" t="n">
+        <v>8</v>
+      </c>
+      <c r="E47" s="20" t="inlineStr">
+        <is>
+          <t>Chemistry</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="27" t="inlineStr">
+        <is>
+          <t>IT (3 students)</t>
+        </is>
+      </c>
+      <c r="B49" s="11" t="n"/>
+      <c r="C49" s="11" t="n"/>
+      <c r="D49" s="11" t="n"/>
+      <c r="E49" s="11" t="n"/>
+    </row>
+    <row r="50">
+      <c r="A50" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="B50" s="8" t="inlineStr">
+        <is>
+          <t>Parviz</t>
+        </is>
+      </c>
+      <c r="C50" s="9" t="inlineStr">
+        <is>
+          <t>9-A</t>
+        </is>
+      </c>
+      <c r="D50" s="3" t="n">
+        <v>9</v>
+      </c>
+      <c r="E50" s="21" t="inlineStr">
+        <is>
+          <t>IT</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="12" t="n">
+        <v>2</v>
+      </c>
+      <c r="B51" s="13" t="inlineStr">
+        <is>
+          <t>Sharipov Abdulaziz</t>
+        </is>
+      </c>
+      <c r="C51" s="14" t="inlineStr">
+        <is>
+          <t>9-A</t>
+        </is>
+      </c>
+      <c r="D51" s="4" t="n">
+        <v>9</v>
+      </c>
+      <c r="E51" s="21" t="inlineStr">
+        <is>
+          <t>IT</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="7" t="n">
+        <v>3</v>
+      </c>
+      <c r="B52" s="8" t="inlineStr">
+        <is>
+          <t>Xudoynazarova Nodira</t>
+        </is>
+      </c>
+      <c r="C52" s="9" t="inlineStr">
+        <is>
+          <t>10-B</t>
+        </is>
+      </c>
+      <c r="D52" s="3" t="n">
+        <v>10</v>
+      </c>
+      <c r="E52" s="21" t="inlineStr">
+        <is>
+          <t>IT</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="28" t="inlineStr">
+        <is>
+          <t>History (2 students)</t>
+        </is>
+      </c>
+      <c r="B54" s="11" t="n"/>
+      <c r="C54" s="11" t="n"/>
+      <c r="D54" s="11" t="n"/>
+      <c r="E54" s="11" t="n"/>
+    </row>
+    <row r="55">
+      <c r="A55" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="B55" s="8" t="inlineStr">
+        <is>
+          <t>Ziyodulla</t>
+        </is>
+      </c>
+      <c r="C55" s="9" t="inlineStr">
+        <is>
+          <t>8-G</t>
+        </is>
+      </c>
+      <c r="D55" s="3" t="n">
+        <v>8</v>
+      </c>
+      <c r="E55" s="19" t="inlineStr">
+        <is>
+          <t>History</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" s="12" t="n">
+        <v>2</v>
+      </c>
+      <c r="B56" s="13" t="inlineStr">
+        <is>
+          <t>Oktambaeva Nozima</t>
+        </is>
+      </c>
+      <c r="C56" s="14" t="inlineStr">
+        <is>
+          <t>9-G</t>
+        </is>
+      </c>
+      <c r="D56" s="4" t="n">
+        <v>9</v>
+      </c>
+      <c r="E56" s="19" t="inlineStr">
+        <is>
+          <t>History</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" s="29" t="inlineStr">
+        <is>
+          <t>Not Assigned (2 students)</t>
+        </is>
+      </c>
+      <c r="B58" s="11" t="n"/>
+      <c r="C58" s="11" t="n"/>
+      <c r="D58" s="11" t="n"/>
+      <c r="E58" s="11" t="n"/>
+    </row>
+    <row r="59">
+      <c r="A59" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="B59" s="8" t="inlineStr">
+        <is>
+          <t>Abdurashidova Mavludaxon</t>
+        </is>
+      </c>
+      <c r="C59" s="9" t="inlineStr">
+        <is>
+          <t>8-P</t>
+        </is>
+      </c>
+      <c r="D59" s="3" t="n">
+        <v>8</v>
+      </c>
+      <c r="E59" s="30" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" s="7" t="n">
+        <v>2</v>
+      </c>
+      <c r="B60" s="8" t="inlineStr">
+        <is>
+          <t>Islomov Xondamir</t>
+        </is>
+      </c>
+      <c r="C60" s="9" t="inlineStr">
+        <is>
+          <t>10-A</t>
+        </is>
+      </c>
+      <c r="D60" s="3" t="n">
+        <v>10</v>
+      </c>
+      <c r="E60" s="30" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" s="31" t="inlineStr">
+        <is>
+          <t>Subject Summary</t>
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" s="2" t="inlineStr">
+        <is>
+          <t>Subject</t>
+        </is>
+      </c>
+      <c r="B63" s="2" t="inlineStr">
+        <is>
+          <t>Students</t>
+        </is>
+      </c>
+      <c r="C63" s="2" t="inlineStr">
+        <is>
+          <t>Color</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" s="8" t="inlineStr">
+        <is>
+          <t>Mathematics</t>
+        </is>
+      </c>
+      <c r="B64" s="3" t="n">
+        <v>15</v>
+      </c>
+      <c r="C64" s="32" t="n"/>
+    </row>
+    <row r="65">
+      <c r="A65" s="8" t="inlineStr">
+        <is>
+          <t>Physics</t>
+        </is>
+      </c>
+      <c r="B65" s="3" t="n">
+        <v>6</v>
+      </c>
+      <c r="C65" s="33" t="n"/>
+    </row>
+    <row r="66">
+      <c r="A66" s="8" t="inlineStr">
+        <is>
+          <t>English</t>
+        </is>
+      </c>
+      <c r="B66" s="3" t="n">
+        <v>8</v>
+      </c>
+      <c r="C66" s="34" t="n"/>
+    </row>
+    <row r="67">
+      <c r="A67" s="8" t="inlineStr">
+        <is>
+          <t>Biology</t>
+        </is>
+      </c>
+      <c r="B67" s="3" t="n">
+        <v>4</v>
+      </c>
+      <c r="C67" s="35" t="n"/>
+    </row>
+    <row r="68">
+      <c r="A68" s="8" t="inlineStr">
+        <is>
+          <t>Chemistry</t>
+        </is>
+      </c>
+      <c r="B68" s="3" t="n">
+        <v>2</v>
+      </c>
+      <c r="C68" s="36" t="n"/>
+    </row>
+    <row r="69">
+      <c r="A69" s="8" t="inlineStr">
+        <is>
+          <t>IT</t>
+        </is>
+      </c>
+      <c r="B69" s="3" t="n">
+        <v>3</v>
+      </c>
+      <c r="C69" s="37" t="n"/>
+    </row>
+    <row r="70">
+      <c r="A70" s="8" t="inlineStr">
+        <is>
+          <t>History</t>
+        </is>
+      </c>
+      <c r="B70" s="3" t="n">
+        <v>2</v>
+      </c>
+      <c r="C70" s="38" t="n"/>
+    </row>
+    <row r="71">
+      <c r="A71" s="39" t="inlineStr">
+        <is>
+          <t>Not Assigned</t>
+        </is>
+      </c>
+      <c r="B71" s="3" t="n">
+        <v>2</v>
+      </c>
+      <c r="C71" s="40" t="n"/>
+    </row>
+    <row r="72">
+      <c r="A72" s="41" t="inlineStr">
+        <is>
+          <t>TOTAL</t>
+        </is>
+      </c>
+      <c r="B72" s="5" t="n">
+        <v>42</v>
+      </c>
+      <c r="C72" s="42" t="n"/>
+    </row>
+  </sheetData>
+  <mergeCells count="10">
+    <mergeCell ref="A21:E21"/>
+    <mergeCell ref="A39:E39"/>
+    <mergeCell ref="A29:E29"/>
+    <mergeCell ref="A4:E4"/>
+    <mergeCell ref="A62:E62"/>
+    <mergeCell ref="A54:E54"/>
+    <mergeCell ref="A49:E49"/>
+    <mergeCell ref="A1:E1"/>
+    <mergeCell ref="A45:E45"/>
+    <mergeCell ref="A58:E58"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>